<commit_message>
Remove o CNPJ da base, das telas e do relatório da folha
A empresa passa a ser identificada só pela coluna EMPRESA. Modelos
de importação (Excel e CSV) atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hd9ZfxUESV4QtaD7RvPDpu
</commit_message>
<xml_diff>
--- a/public/exemplos/base-elegibilidade-modelo.xlsx
+++ b/public/exemplos/base-elegibilidade-modelo.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C31"/>
   <cols>
     <col min="1" max="1" width="44.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -500,224 +500,212 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CNPJ</v>
+        <v>UNIDADE</v>
       </c>
       <c r="B12" t="str">
         <v>Não*</v>
       </c>
       <c r="C12" t="str">
-        <v>CNPJ da empresa (relatório da folha).</v>
+        <v>Unidade/lotação (filtros e relatório da folha).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>UNIDADE</v>
+        <v>DATA_ADMISSAO</v>
       </c>
       <c r="B13" t="str">
-        <v>Não*</v>
+        <v>Recomendada</v>
       </c>
       <c r="C13" t="str">
-        <v>Unidade/lotação (filtros e relatório da folha).</v>
+        <v>Usada para definir sucedido quando a coluna SUCEDIDO estiver vazia (até 31/12/2011 = sucedido).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>DATA_ADMISSAO</v>
+        <v>SUCEDIDO</v>
       </c>
       <c r="B14" t="str">
         <v>Recomendada</v>
       </c>
       <c r="C14" t="str">
-        <v>Usada para definir sucedido quando a coluna SUCEDIDO estiver vazia (até 31/12/2011 = sucedido).</v>
+        <v>S = sucedido, N = não sucedido. Define os limites de educacional e creche e o direito de pai/mãe no medicamento.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SUCEDIDO</v>
+        <v>DATA_DESLIGAMENTO</v>
       </c>
       <c r="B15" t="str">
-        <v>Recomendada</v>
+        <v>Não</v>
       </c>
       <c r="C15" t="str">
-        <v>S = sucedido, N = não sucedido. Define os limites de educacional e creche e o direito de pai/mãe no medicamento.</v>
+        <v>Se preenchida, bloqueia documentos com data posterior ao desligamento.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>DATA_DESLIGAMENTO</v>
+        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
       </c>
       <c r="B16" t="str">
         <v>Não</v>
       </c>
       <c r="C16" t="str">
-        <v>Se preenchida, bloqueia documentos com data posterior ao desligamento.</v>
+        <v>Vazio = segue a regra do benefício (recomendado). N = bloqueia o benefício para o colaborador e toda a família. S = sem efeito extra para o titular.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Não</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Vazio = segue a regra do benefício (recomendado). N = bloqueia o benefício para o colaborador e toda a família. S = sem efeito extra para o titular.</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>ABA DEPENDENTES</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Obrigatória?</v>
+      </c>
+      <c r="C18" t="str">
+        <v>O que preencher</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ABA DEPENDENTES</v>
+        <v>CPF_TITULAR</v>
       </c>
       <c r="B19" t="str">
-        <v>Obrigatória?</v>
+        <v>Sim</v>
       </c>
       <c r="C19" t="str">
-        <v>O que preencher</v>
+        <v>CPF do colaborador (precisa existir na aba Colaboradores).</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CPF_TITULAR</v>
+        <v>NOME</v>
       </c>
       <c r="B20" t="str">
         <v>Sim</v>
       </c>
       <c r="C20" t="str">
-        <v>CPF do colaborador (precisa existir na aba Colaboradores).</v>
+        <v>Nome completo do dependente.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>NOME</v>
+        <v>CPF</v>
       </c>
       <c r="B21" t="str">
-        <v>Sim</v>
+        <v>Recomendada</v>
       </c>
       <c r="C21" t="str">
-        <v>Nome completo do dependente.</v>
+        <v>CPF do dependente. Identifica o mesmo dependente entre os meses (sem CPF, usa nome + nascimento).</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CPF</v>
+        <v>PARENTESCO</v>
       </c>
       <c r="B22" t="str">
-        <v>Recomendada</v>
+        <v>Sim</v>
       </c>
       <c r="C22" t="str">
-        <v>CPF do dependente. Identifica o mesmo dependente entre os meses (sem CPF, usa nome + nascimento).</v>
+        <v>Cônjuge (ou Companheiro), Filho/Filha, Enteado/Enteada, Neto/Neta (com tutela), Tutelado, Pai, Mãe.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>PARENTESCO</v>
+        <v>DATA_NASCIMENTO</v>
       </c>
       <c r="B23" t="str">
-        <v>Sim</v>
+        <v>Sim**</v>
       </c>
       <c r="C23" t="str">
-        <v>Cônjuge (ou Companheiro), Filho/Filha, Enteado/Enteada, Neto/Neta (com tutela), Tutelado, Pai, Mãe.</v>
+        <v>Obrigatória para educacional (7 a 17 anos) e creche (6 meses a 6 anos).</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>DATA_NASCIMENTO</v>
+        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
       </c>
       <c r="B24" t="str">
-        <v>Sim**</v>
+        <v>Não</v>
       </c>
       <c r="C24" t="str">
-        <v>Obrigatória para educacional (7 a 17 anos) e creche (6 meses a 6 anos).</v>
+        <v>Vazio = segue a regra (parentesco e idade). S = libera mesmo fora da regra (exceção aprovada pelo RH). N = bloqueia este dependente no benefício.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Não</v>
-      </c>
-      <c r="C25" t="str">
-        <v>Vazio = segue a regra (parentesco e idade). S = libera mesmo fora da regra (exceção aprovada pelo RH). N = bloqueia este dependente no benefício.</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v/>
+        <v>* Não bloqueia a importação, mas deixa o relatório da folha incompleto.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>* Não bloqueia a importação, mas deixa o relatório da folha incompleto.</v>
+        <v>** Sem a data, o dependente não aparece para educacional e creche (a menos que a coluna do benefício esteja com S).</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>** Sem a data, o dependente não aparece para educacional e creche (a menos que a coluna do benefício esteja com S).</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>MODOS DE IMPORTAÇÃO</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>MODOS DE IMPORTAÇÃO</v>
+        <v>Adicionar / atualizar</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v>Inclui novos e atualiza quem já existe. Ninguém perde acesso.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Adicionar / atualizar</v>
+        <v>Substituir base</v>
       </c>
       <c r="B31" t="str">
         <v/>
       </c>
       <c r="C31" t="str">
-        <v>Inclui novos e atualiza quem já existe. Ninguém perde acesso.</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Substituir base</v>
-      </c>
-      <c r="B32" t="str">
-        <v/>
-      </c>
-      <c r="C32" t="str">
         <v>Recomendado na carga mensal completa: quem não estiver na planilha perde o acesso (desligados). O histórico de solicitações é mantido.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="30.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="19.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
     <col min="11" max="11" width="13.83203125" customWidth="1"/>
-    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="9.83203125" customWidth="1"/>
     <col min="13" max="13" width="9.83203125" customWidth="1"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -737,30 +725,27 @@
         <v>EMPRESA</v>
       </c>
       <c r="F1" s="1" t="str">
-        <v>CNPJ</v>
+        <v>UNIDADE</v>
       </c>
       <c r="G1" s="1" t="str">
-        <v>UNIDADE</v>
+        <v>DATA_ADMISSAO</v>
       </c>
       <c r="H1" s="1" t="str">
-        <v>DATA_ADMISSAO</v>
+        <v>SUCEDIDO</v>
       </c>
       <c r="I1" s="1" t="str">
-        <v>SUCEDIDO</v>
+        <v>DATA_DESLIGAMENTO</v>
       </c>
       <c r="J1" s="1" t="str">
-        <v>DATA_DESLIGAMENTO</v>
+        <v>MEDICAMENTO</v>
       </c>
       <c r="K1" s="1" t="str">
-        <v>MEDICAMENTO</v>
+        <v>EDUCACIONAL</v>
       </c>
       <c r="L1" s="1" t="str">
-        <v>EDUCACIONAL</v>
+        <v>CRECHE</v>
       </c>
       <c r="M1" s="1" t="str">
-        <v>CRECHE</v>
-      </c>
-      <c r="N1" s="1" t="str">
         <v>OCULOS</v>
       </c>
     </row>
@@ -781,16 +766,16 @@
         <v>Âmbar Energia</v>
       </c>
       <c r="F2" s="1" t="str">
-        <v>00.000.000/0001-00</v>
+        <v>Cuiabá</v>
       </c>
       <c r="G2" s="1" t="str">
-        <v>Cuiabá</v>
+        <v>15/03/2008</v>
       </c>
       <c r="H2" s="1" t="str">
-        <v>15/03/2008</v>
+        <v>S</v>
       </c>
       <c r="I2" s="1" t="str">
-        <v>S</v>
+        <v/>
       </c>
       <c r="J2" s="1" t="str">
         <v/>
@@ -802,9 +787,6 @@
         <v/>
       </c>
       <c r="M2" s="1" t="str">
-        <v/>
-      </c>
-      <c r="N2" s="1" t="str">
         <v/>
       </c>
     </row>
@@ -825,16 +807,16 @@
         <v>Fluxus</v>
       </c>
       <c r="F3" s="1" t="str">
-        <v>00.000.000/0002-00</v>
+        <v>Campo Grande</v>
       </c>
       <c r="G3" s="1" t="str">
-        <v>Campo Grande</v>
+        <v>03/02/2025</v>
       </c>
       <c r="H3" s="1" t="str">
-        <v>03/02/2025</v>
+        <v>N</v>
       </c>
       <c r="I3" s="1" t="str">
-        <v>N</v>
+        <v/>
       </c>
       <c r="J3" s="1" t="str">
         <v/>
@@ -846,15 +828,12 @@
         <v/>
       </c>
       <c r="M3" s="1" t="str">
-        <v/>
-      </c>
-      <c r="N3" s="1" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remove a empresa da base, das telas e do relatório da folha
O painel do RH passa a mostrar o resumo por unidade. Modelos de
importação (Excel e CSV) atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hd9ZfxUESV4QtaD7RvPDpu
</commit_message>
<xml_diff>
--- a/public/exemplos/base-elegibilidade-modelo.xlsx
+++ b/public/exemplos/base-elegibilidade-modelo.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="44.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -489,223 +489,211 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EMPRESA</v>
+        <v>UNIDADE</v>
       </c>
       <c r="B11" t="str">
         <v>Não*</v>
       </c>
       <c r="C11" t="str">
-        <v>Empresa do grupo (filtros e relatório da folha).</v>
+        <v>Unidade/lotação (filtros e relatório da folha).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>UNIDADE</v>
+        <v>DATA_ADMISSAO</v>
       </c>
       <c r="B12" t="str">
-        <v>Não*</v>
+        <v>Recomendada</v>
       </c>
       <c r="C12" t="str">
-        <v>Unidade/lotação (filtros e relatório da folha).</v>
+        <v>Usada para definir sucedido quando a coluna SUCEDIDO estiver vazia (até 31/12/2011 = sucedido).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>DATA_ADMISSAO</v>
+        <v>SUCEDIDO</v>
       </c>
       <c r="B13" t="str">
         <v>Recomendada</v>
       </c>
       <c r="C13" t="str">
-        <v>Usada para definir sucedido quando a coluna SUCEDIDO estiver vazia (até 31/12/2011 = sucedido).</v>
+        <v>S = sucedido, N = não sucedido. Define os limites de educacional e creche e o direito de pai/mãe no medicamento.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SUCEDIDO</v>
+        <v>DATA_DESLIGAMENTO</v>
       </c>
       <c r="B14" t="str">
-        <v>Recomendada</v>
+        <v>Não</v>
       </c>
       <c r="C14" t="str">
-        <v>S = sucedido, N = não sucedido. Define os limites de educacional e creche e o direito de pai/mãe no medicamento.</v>
+        <v>Se preenchida, bloqueia documentos com data posterior ao desligamento.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>DATA_DESLIGAMENTO</v>
+        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
       </c>
       <c r="B15" t="str">
         <v>Não</v>
       </c>
       <c r="C15" t="str">
-        <v>Se preenchida, bloqueia documentos com data posterior ao desligamento.</v>
+        <v>Vazio = segue a regra do benefício (recomendado). N = bloqueia o benefício para o colaborador e toda a família. S = sem efeito extra para o titular.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Não</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Vazio = segue a regra do benefício (recomendado). N = bloqueia o benefício para o colaborador e toda a família. S = sem efeito extra para o titular.</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>ABA DEPENDENTES</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Obrigatória?</v>
+      </c>
+      <c r="C17" t="str">
+        <v>O que preencher</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ABA DEPENDENTES</v>
+        <v>CPF_TITULAR</v>
       </c>
       <c r="B18" t="str">
-        <v>Obrigatória?</v>
+        <v>Sim</v>
       </c>
       <c r="C18" t="str">
-        <v>O que preencher</v>
+        <v>CPF do colaborador (precisa existir na aba Colaboradores).</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CPF_TITULAR</v>
+        <v>NOME</v>
       </c>
       <c r="B19" t="str">
         <v>Sim</v>
       </c>
       <c r="C19" t="str">
-        <v>CPF do colaborador (precisa existir na aba Colaboradores).</v>
+        <v>Nome completo do dependente.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NOME</v>
+        <v>CPF</v>
       </c>
       <c r="B20" t="str">
-        <v>Sim</v>
+        <v>Recomendada</v>
       </c>
       <c r="C20" t="str">
-        <v>Nome completo do dependente.</v>
+        <v>CPF do dependente. Identifica o mesmo dependente entre os meses (sem CPF, usa nome + nascimento).</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CPF</v>
+        <v>PARENTESCO</v>
       </c>
       <c r="B21" t="str">
-        <v>Recomendada</v>
+        <v>Sim</v>
       </c>
       <c r="C21" t="str">
-        <v>CPF do dependente. Identifica o mesmo dependente entre os meses (sem CPF, usa nome + nascimento).</v>
+        <v>Cônjuge (ou Companheiro), Filho/Filha, Enteado/Enteada, Neto/Neta (com tutela), Tutelado, Pai, Mãe.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>PARENTESCO</v>
+        <v>DATA_NASCIMENTO</v>
       </c>
       <c r="B22" t="str">
-        <v>Sim</v>
+        <v>Sim**</v>
       </c>
       <c r="C22" t="str">
-        <v>Cônjuge (ou Companheiro), Filho/Filha, Enteado/Enteada, Neto/Neta (com tutela), Tutelado, Pai, Mãe.</v>
+        <v>Obrigatória para educacional (7 a 17 anos) e creche (6 meses a 6 anos).</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>DATA_NASCIMENTO</v>
+        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
       </c>
       <c r="B23" t="str">
-        <v>Sim**</v>
+        <v>Não</v>
       </c>
       <c r="C23" t="str">
-        <v>Obrigatória para educacional (7 a 17 anos) e creche (6 meses a 6 anos).</v>
+        <v>Vazio = segue a regra (parentesco e idade). S = libera mesmo fora da regra (exceção aprovada pelo RH). N = bloqueia este dependente no benefício.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Não</v>
-      </c>
-      <c r="C24" t="str">
-        <v>Vazio = segue a regra (parentesco e idade). S = libera mesmo fora da regra (exceção aprovada pelo RH). N = bloqueia este dependente no benefício.</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v>* Não bloqueia a importação, mas deixa o relatório da folha incompleto.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>* Não bloqueia a importação, mas deixa o relatório da folha incompleto.</v>
+        <v>** Sem a data, o dependente não aparece para educacional e creche (a menos que a coluna do benefício esteja com S).</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>** Sem a data, o dependente não aparece para educacional e creche (a menos que a coluna do benefício esteja com S).</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v/>
+        <v>MODOS DE IMPORTAÇÃO</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>MODOS DE IMPORTAÇÃO</v>
+        <v>Adicionar / atualizar</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v>Inclui novos e atualiza quem já existe. Ninguém perde acesso.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Adicionar / atualizar</v>
+        <v>Substituir base</v>
       </c>
       <c r="B30" t="str">
         <v/>
       </c>
       <c r="C30" t="str">
-        <v>Inclui novos e atualiza quem já existe. Ninguém perde acesso.</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>Substituir base</v>
-      </c>
-      <c r="B31" t="str">
-        <v/>
-      </c>
-      <c r="C31" t="str">
         <v>Recomendado na carga mensal completa: quem não estiver na planilha perde o acesso (desligados). O histórico de solicitações é mantido.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:L3"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="30.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="19.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
     <col min="10" max="10" width="13.83203125" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" customWidth="1"/>
     <col min="12" max="12" width="9.83203125" customWidth="1"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -722,30 +710,27 @@
         <v>EMAIL</v>
       </c>
       <c r="E1" s="1" t="str">
-        <v>EMPRESA</v>
+        <v>UNIDADE</v>
       </c>
       <c r="F1" s="1" t="str">
-        <v>UNIDADE</v>
+        <v>DATA_ADMISSAO</v>
       </c>
       <c r="G1" s="1" t="str">
-        <v>DATA_ADMISSAO</v>
+        <v>SUCEDIDO</v>
       </c>
       <c r="H1" s="1" t="str">
-        <v>SUCEDIDO</v>
+        <v>DATA_DESLIGAMENTO</v>
       </c>
       <c r="I1" s="1" t="str">
-        <v>DATA_DESLIGAMENTO</v>
+        <v>MEDICAMENTO</v>
       </c>
       <c r="J1" s="1" t="str">
-        <v>MEDICAMENTO</v>
+        <v>EDUCACIONAL</v>
       </c>
       <c r="K1" s="1" t="str">
-        <v>EDUCACIONAL</v>
+        <v>CRECHE</v>
       </c>
       <c r="L1" s="1" t="str">
-        <v>CRECHE</v>
-      </c>
-      <c r="M1" s="1" t="str">
         <v>OCULOS</v>
       </c>
     </row>
@@ -763,16 +748,16 @@
         <v>maria.souza@empresa.com.br</v>
       </c>
       <c r="E2" s="1" t="str">
-        <v>Âmbar Energia</v>
+        <v>Cuiabá</v>
       </c>
       <c r="F2" s="1" t="str">
-        <v>Cuiabá</v>
+        <v>15/03/2008</v>
       </c>
       <c r="G2" s="1" t="str">
-        <v>15/03/2008</v>
+        <v>S</v>
       </c>
       <c r="H2" s="1" t="str">
-        <v>S</v>
+        <v/>
       </c>
       <c r="I2" s="1" t="str">
         <v/>
@@ -784,9 +769,6 @@
         <v/>
       </c>
       <c r="L2" s="1" t="str">
-        <v/>
-      </c>
-      <c r="M2" s="1" t="str">
         <v/>
       </c>
     </row>
@@ -804,16 +786,16 @@
         <v>joao.pereira@empresa.com.br</v>
       </c>
       <c r="E3" s="1" t="str">
-        <v>Fluxus</v>
+        <v>Campo Grande</v>
       </c>
       <c r="F3" s="1" t="str">
-        <v>Campo Grande</v>
+        <v>03/02/2025</v>
       </c>
       <c r="G3" s="1" t="str">
-        <v>03/02/2025</v>
+        <v>N</v>
       </c>
       <c r="H3" s="1" t="str">
-        <v>N</v>
+        <v/>
       </c>
       <c r="I3" s="1" t="str">
         <v/>
@@ -825,15 +807,12 @@
         <v/>
       </c>
       <c r="L3" s="1" t="str">
-        <v/>
-      </c>
-      <c r="M3" s="1" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Importação aceita a planilha de colaboradores do RH como ela sai
Cabeçalhos com acentos, espaços e conectivos (Matrícula, Data de
Admissão), Filial como unidade e '-' no e-mail tratado como vazio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hd9ZfxUESV4QtaD7RvPDpu
</commit_message>
<xml_diff>
--- a/public/exemplos/base-elegibilidade-modelo.xlsx
+++ b/public/exemplos/base-elegibilidade-modelo.xlsx
@@ -424,7 +424,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Datas no formato DD/MM/AAAA (ou como data do Excel). CPF com ou sem pontuação (zeros à esquerda perdidos pelo Excel são recuperados).</v>
+        <v>Datas no formato DD/MM/AAAA (ou como data do Excel). CPF com ou sem pontuação (zeros à esquerda perdidos pelo Excel são recuperados). Os cabeçalhos podem ter acentos e espaços (ex.: Matrícula, Data de Admissão, Filial).</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         <v>Não</v>
       </c>
       <c r="C10" t="str">
-        <v>Para os avisos de envio, aprovação e reprovação.</v>
+        <v>Para os avisos de envio, aprovação e reprovação. Pode ficar vazio ou com "-".</v>
       </c>
     </row>
     <row r="11">
@@ -495,7 +495,7 @@
         <v>Não*</v>
       </c>
       <c r="C11" t="str">
-        <v>Unidade/lotação (filtros e relatório da folha).</v>
+        <v>Unidade/lotação (filtros e relatório da folha). Também aceita o cabeçalho FILIAL ou LOTAÇÃO.</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Novo benefício: Reembolso Material Escolar/Uniforme
- Filhos de 7 a 17 anos; R$ 1.467,26 (sucedido) / R$ 1.200,00 (não sucedido) por dependente
- Solicitado somente em fevereiro e julho: um reembolso por dependente em cada mês,
  sem acumular saldo entre as janelas; reprovado libera novo envio
- Bloqueio no envio e na aprovação do RH, com a próxima janela indicada no portal
- Coluna MATERIAL na importação da base e nos modelos; limites editáveis na Administração
- Home, portal, guia de acesso (PDF) e README atualizados; testes das regras

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hd9ZfxUESV4QtaD7RvPDpu
</commit_message>
<xml_diff>
--- a/public/exemplos/base-elegibilidade-modelo.xlsx
+++ b/public/exemplos/base-elegibilidade-modelo.xlsx
@@ -517,7 +517,7 @@
         <v>Recomendada</v>
       </c>
       <c r="C13" t="str">
-        <v>S = sucedido, N = não sucedido. Define os limites de educacional e creche e o direito de pai/mãe no medicamento.</v>
+        <v>S = sucedido, N = não sucedido. Define os limites de educacional, creche e material escolar/uniforme e o direito de pai/mãe no medicamento.</v>
       </c>
     </row>
     <row r="14">
@@ -533,7 +533,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
+        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS / MATERIAL</v>
       </c>
       <c r="B15" t="str">
         <v>Não</v>
@@ -610,12 +610,12 @@
         <v>Sim**</v>
       </c>
       <c r="C22" t="str">
-        <v>Obrigatória para educacional (7 a 17 anos) e creche (6 meses a 6 anos).</v>
+        <v>Obrigatória para educacional e material escolar/uniforme (7 a 17 anos) e creche (6 meses a 6 anos).</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS</v>
+        <v>MEDICAMENTO / EDUCACIONAL / CRECHE / OCULOS / MATERIAL</v>
       </c>
       <c r="B23" t="str">
         <v>Não</v>
@@ -636,7 +636,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>** Sem a data, o dependente não aparece para educacional e creche (a menos que a coluna do benefício esteja com S).</v>
+        <v>** Sem a data, o dependente não aparece para educacional, creche e material escolar/uniforme (a menos que a coluna do benefício esteja com S).</v>
       </c>
     </row>
     <row r="27">
@@ -680,7 +680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -694,6 +694,7 @@
     <col min="10" max="10" width="13.83203125" customWidth="1"/>
     <col min="11" max="11" width="9.83203125" customWidth="1"/>
     <col min="12" max="12" width="9.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -733,6 +734,9 @@
       <c r="L1" s="1" t="str">
         <v>OCULOS</v>
       </c>
+      <c r="M1" s="1" t="str">
+        <v>MATERIAL</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
@@ -771,6 +775,9 @@
       <c r="L2" s="1" t="str">
         <v/>
       </c>
+      <c r="M2" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
@@ -809,17 +816,20 @@
       <c r="L3" s="1" t="str">
         <v/>
       </c>
+      <c r="M3" s="1" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -830,6 +840,7 @@
     <col min="7" max="7" width="13.83203125" customWidth="1"/>
     <col min="8" max="8" width="9.83203125" customWidth="1"/>
     <col min="9" max="9" width="9.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -860,6 +871,9 @@
       <c r="I1" s="1" t="str">
         <v>OCULOS</v>
       </c>
+      <c r="J1" s="1" t="str">
+        <v>MATERIAL</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
@@ -889,6 +903,9 @@
       <c r="I2" s="1" t="str">
         <v/>
       </c>
+      <c r="J2" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
@@ -918,6 +935,9 @@
       <c r="I3" s="1" t="str">
         <v/>
       </c>
+      <c r="J3" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
@@ -947,6 +967,9 @@
       <c r="I4" s="1" t="str">
         <v/>
       </c>
+      <c r="J4" s="1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
@@ -976,10 +999,13 @@
       <c r="I5" s="1" t="str">
         <v/>
       </c>
+      <c r="J5" s="1" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>